<commit_message>
[FEATURE] Added file and items validation.
</commit_message>
<xml_diff>
--- a/src/microservices/notifications/static/Plantilla Dependencias.xlsx
+++ b/src/microservices/notifications/static/Plantilla Dependencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BitBang\Projects\CaliMovilidad\cali-mobility-backend\src\microservices\notifications\static\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TBBC\Proyectos\Cali Movilidad\cali-mobility-backend\src\microservices\notifications\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53BBE4F-DB95-473C-B19F-3E6497C31F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFD59E8-DED4-4653-B4E2-C4429E65075D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -124,57 +124,17 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{F7A4D92E-3B1F-4389-8792-03A92E948B4F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Nota sobre Teléfono Dependencia:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Hace referencia al número de teléfono de contacto de cada dependencia. Solo se debe configurar un único número por dependencia.
-- Debe ser un número telefónico de Colombia fijo o móvil.
-- Debe ser un número de 10 cifras.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <i/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Este campo es obligatorio.</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>ID Único</t>
   </si>
   <si>
     <t>Nombre Dependencia</t>
-  </si>
-  <si>
-    <t>Teléfono Dependencia</t>
   </si>
   <si>
     <t>Primer ejemplo de Dependencia de prueba</t>
@@ -527,44 +487,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>3101230123</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>6011230123</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>